<commit_message>
Billable hours 5.5 -> 5 per BA across schedule + all deliverables
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feel_Free_Summer2026_Route_Plan_INTERNAL.xlsx
+++ b/Feel_Free_Summer2026_Route_Plan_INTERNAL.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Master Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MIA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FTL" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TPA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="AUS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SAT" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="PHX" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FTL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAT" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHX" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Schedule'!$A$1:$P$250</definedName>
@@ -732,7 +732,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>2 BAs/shift · 5.5 billable hrs/BA</t>
+          <t>2 BAs/shift · 5 billable hrs/BA</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>249 shifts · 498 BA-slots · 1370 BA-hours</t>
+          <t>249 shifts · 498 BA-slots · 1245 BA-hours</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>245</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>245</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>245</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>255</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>255</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1205,7 +1205,7 @@
         <v>2</v>
       </c>
       <c r="O2" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P2" s="15" t="inlineStr"/>
     </row>
@@ -1277,7 +1277,7 @@
         <v>2</v>
       </c>
       <c r="O3" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P3" s="15" t="inlineStr"/>
     </row>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="O4" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P4" s="17" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="O5" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P5" s="15" t="inlineStr"/>
     </row>
@@ -1497,7 +1497,7 @@
         <v>2</v>
       </c>
       <c r="O6" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P6" s="15" t="inlineStr"/>
     </row>
@@ -1569,7 +1569,7 @@
         <v>2</v>
       </c>
       <c r="O7" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P7" s="15" t="inlineStr"/>
     </row>
@@ -1641,7 +1641,7 @@
         <v>2</v>
       </c>
       <c r="O8" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P8" s="17" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         <v>2</v>
       </c>
       <c r="O9" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P9" s="15" t="inlineStr"/>
     </row>
@@ -1789,7 +1789,7 @@
         <v>2</v>
       </c>
       <c r="O10" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P10" s="15" t="inlineStr"/>
     </row>
@@ -1861,7 +1861,7 @@
         <v>2</v>
       </c>
       <c r="O11" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P11" s="15" t="inlineStr"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>2</v>
       </c>
       <c r="O12" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P12" s="15" t="inlineStr"/>
     </row>
@@ -2005,7 +2005,7 @@
         <v>2</v>
       </c>
       <c r="O13" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P13" s="15" t="inlineStr"/>
     </row>
@@ -2077,7 +2077,7 @@
         <v>2</v>
       </c>
       <c r="O14" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P14" s="15" t="inlineStr"/>
     </row>
@@ -2149,7 +2149,7 @@
         <v>2</v>
       </c>
       <c r="O15" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P15" s="15" t="inlineStr"/>
     </row>
@@ -2221,7 +2221,7 @@
         <v>2</v>
       </c>
       <c r="O16" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P16" s="15" t="inlineStr"/>
     </row>
@@ -2293,7 +2293,7 @@
         <v>2</v>
       </c>
       <c r="O17" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P17" s="15" t="inlineStr"/>
     </row>
@@ -2365,7 +2365,7 @@
         <v>2</v>
       </c>
       <c r="O18" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P18" s="15" t="inlineStr"/>
     </row>
@@ -2437,7 +2437,7 @@
         <v>2</v>
       </c>
       <c r="O19" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P19" s="15" t="inlineStr"/>
     </row>
@@ -2509,7 +2509,7 @@
         <v>2</v>
       </c>
       <c r="O20" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P20" s="15" t="inlineStr"/>
     </row>
@@ -2581,7 +2581,7 @@
         <v>2</v>
       </c>
       <c r="O21" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P21" s="15" t="inlineStr"/>
     </row>
@@ -2653,7 +2653,7 @@
         <v>2</v>
       </c>
       <c r="O22" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P22" s="15" t="inlineStr"/>
     </row>
@@ -2725,7 +2725,7 @@
         <v>2</v>
       </c>
       <c r="O23" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P23" s="15" t="inlineStr"/>
     </row>
@@ -2797,7 +2797,7 @@
         <v>2</v>
       </c>
       <c r="O24" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P24" s="15" t="inlineStr"/>
     </row>
@@ -2869,7 +2869,7 @@
         <v>2</v>
       </c>
       <c r="O25" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P25" s="15" t="inlineStr"/>
     </row>
@@ -2941,7 +2941,7 @@
         <v>2</v>
       </c>
       <c r="O26" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P26" s="15" t="inlineStr"/>
     </row>
@@ -3013,7 +3013,7 @@
         <v>2</v>
       </c>
       <c r="O27" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P27" s="15" t="inlineStr"/>
     </row>
@@ -3085,7 +3085,7 @@
         <v>2</v>
       </c>
       <c r="O28" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P28" s="15" t="inlineStr"/>
     </row>
@@ -3157,7 +3157,7 @@
         <v>2</v>
       </c>
       <c r="O29" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P29" s="15" t="inlineStr"/>
     </row>
@@ -3229,7 +3229,7 @@
         <v>2</v>
       </c>
       <c r="O30" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P30" s="15" t="inlineStr"/>
     </row>
@@ -3301,7 +3301,7 @@
         <v>2</v>
       </c>
       <c r="O31" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P31" s="15" t="inlineStr"/>
     </row>
@@ -3373,7 +3373,7 @@
         <v>2</v>
       </c>
       <c r="O32" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P32" s="15" t="inlineStr"/>
     </row>
@@ -3445,7 +3445,7 @@
         <v>2</v>
       </c>
       <c r="O33" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P33" s="15" t="inlineStr"/>
     </row>
@@ -3517,7 +3517,7 @@
         <v>2</v>
       </c>
       <c r="O34" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P34" s="15" t="inlineStr"/>
     </row>
@@ -3589,7 +3589,7 @@
         <v>2</v>
       </c>
       <c r="O35" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P35" s="15" t="inlineStr"/>
     </row>
@@ -3661,7 +3661,7 @@
         <v>2</v>
       </c>
       <c r="O36" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P36" s="15" t="inlineStr"/>
     </row>
@@ -3733,7 +3733,7 @@
         <v>2</v>
       </c>
       <c r="O37" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P37" s="15" t="inlineStr"/>
     </row>
@@ -3805,7 +3805,7 @@
         <v>2</v>
       </c>
       <c r="O38" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P38" s="15" t="inlineStr"/>
     </row>
@@ -3877,7 +3877,7 @@
         <v>2</v>
       </c>
       <c r="O39" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P39" s="15" t="inlineStr"/>
     </row>
@@ -3949,7 +3949,7 @@
         <v>2</v>
       </c>
       <c r="O40" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P40" s="15" t="inlineStr"/>
     </row>
@@ -4021,7 +4021,7 @@
         <v>2</v>
       </c>
       <c r="O41" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P41" s="15" t="inlineStr"/>
     </row>
@@ -4093,7 +4093,7 @@
         <v>2</v>
       </c>
       <c r="O42" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P42" s="15" t="inlineStr"/>
     </row>
@@ -4165,7 +4165,7 @@
         <v>2</v>
       </c>
       <c r="O43" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P43" s="15" t="inlineStr"/>
     </row>
@@ -4237,7 +4237,7 @@
         <v>2</v>
       </c>
       <c r="O44" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P44" s="15" t="inlineStr"/>
     </row>
@@ -4309,7 +4309,7 @@
         <v>2</v>
       </c>
       <c r="O45" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P45" s="15" t="inlineStr"/>
     </row>
@@ -4381,7 +4381,7 @@
         <v>2</v>
       </c>
       <c r="O46" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P46" s="15" t="inlineStr"/>
     </row>
@@ -4453,7 +4453,7 @@
         <v>2</v>
       </c>
       <c r="O47" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P47" s="15" t="inlineStr"/>
     </row>
@@ -4525,7 +4525,7 @@
         <v>2</v>
       </c>
       <c r="O48" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P48" s="15" t="inlineStr"/>
     </row>
@@ -4597,7 +4597,7 @@
         <v>2</v>
       </c>
       <c r="O49" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P49" s="15" t="inlineStr"/>
     </row>
@@ -4669,7 +4669,7 @@
         <v>2</v>
       </c>
       <c r="O50" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P50" s="15" t="inlineStr"/>
     </row>
@@ -4741,7 +4741,7 @@
         <v>2</v>
       </c>
       <c r="O51" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P51" s="15" t="inlineStr"/>
     </row>
@@ -4813,7 +4813,7 @@
         <v>2</v>
       </c>
       <c r="O52" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P52" s="15" t="inlineStr"/>
     </row>
@@ -4885,7 +4885,7 @@
         <v>2</v>
       </c>
       <c r="O53" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P53" s="17" t="inlineStr">
         <is>
@@ -4961,7 +4961,7 @@
         <v>2</v>
       </c>
       <c r="O54" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P54" s="15" t="inlineStr"/>
     </row>
@@ -5033,7 +5033,7 @@
         <v>2</v>
       </c>
       <c r="O55" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P55" s="15" t="inlineStr"/>
     </row>
@@ -5105,7 +5105,7 @@
         <v>2</v>
       </c>
       <c r="O56" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P56" s="15" t="inlineStr"/>
     </row>
@@ -5177,7 +5177,7 @@
         <v>2</v>
       </c>
       <c r="O57" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P57" s="15" t="inlineStr"/>
     </row>
@@ -5249,7 +5249,7 @@
         <v>2</v>
       </c>
       <c r="O58" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P58" s="15" t="inlineStr"/>
     </row>
@@ -5321,7 +5321,7 @@
         <v>2</v>
       </c>
       <c r="O59" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P59" s="15" t="inlineStr"/>
     </row>
@@ -5393,7 +5393,7 @@
         <v>2</v>
       </c>
       <c r="O60" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P60" s="15" t="inlineStr"/>
     </row>
@@ -5465,7 +5465,7 @@
         <v>2</v>
       </c>
       <c r="O61" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P61" s="15" t="inlineStr"/>
     </row>
@@ -5537,7 +5537,7 @@
         <v>2</v>
       </c>
       <c r="O62" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P62" s="15" t="inlineStr"/>
     </row>
@@ -5609,7 +5609,7 @@
         <v>2</v>
       </c>
       <c r="O63" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P63" s="15" t="inlineStr"/>
     </row>
@@ -5681,7 +5681,7 @@
         <v>2</v>
       </c>
       <c r="O64" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P64" s="15" t="inlineStr"/>
     </row>
@@ -5753,7 +5753,7 @@
         <v>2</v>
       </c>
       <c r="O65" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P65" s="15" t="inlineStr"/>
     </row>
@@ -5825,7 +5825,7 @@
         <v>2</v>
       </c>
       <c r="O66" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P66" s="15" t="inlineStr"/>
     </row>
@@ -5897,7 +5897,7 @@
         <v>2</v>
       </c>
       <c r="O67" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P67" s="15" t="inlineStr"/>
     </row>
@@ -5969,7 +5969,7 @@
         <v>2</v>
       </c>
       <c r="O68" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P68" s="15" t="inlineStr"/>
     </row>
@@ -6041,7 +6041,7 @@
         <v>2</v>
       </c>
       <c r="O69" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P69" s="15" t="inlineStr"/>
     </row>
@@ -6113,7 +6113,7 @@
         <v>2</v>
       </c>
       <c r="O70" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P70" s="15" t="inlineStr"/>
     </row>
@@ -6185,7 +6185,7 @@
         <v>2</v>
       </c>
       <c r="O71" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P71" s="15" t="inlineStr"/>
     </row>
@@ -6257,7 +6257,7 @@
         <v>2</v>
       </c>
       <c r="O72" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P72" s="15" t="inlineStr"/>
     </row>
@@ -6329,7 +6329,7 @@
         <v>2</v>
       </c>
       <c r="O73" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P73" s="15" t="inlineStr"/>
     </row>
@@ -6401,7 +6401,7 @@
         <v>2</v>
       </c>
       <c r="O74" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P74" s="15" t="inlineStr"/>
     </row>
@@ -6473,7 +6473,7 @@
         <v>2</v>
       </c>
       <c r="O75" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P75" s="15" t="inlineStr"/>
     </row>
@@ -6545,7 +6545,7 @@
         <v>2</v>
       </c>
       <c r="O76" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P76" s="15" t="inlineStr"/>
     </row>
@@ -6617,7 +6617,7 @@
         <v>2</v>
       </c>
       <c r="O77" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P77" s="15" t="inlineStr"/>
     </row>
@@ -6689,7 +6689,7 @@
         <v>2</v>
       </c>
       <c r="O78" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P78" s="15" t="inlineStr"/>
     </row>
@@ -6761,7 +6761,7 @@
         <v>2</v>
       </c>
       <c r="O79" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P79" s="15" t="inlineStr"/>
     </row>
@@ -6833,7 +6833,7 @@
         <v>2</v>
       </c>
       <c r="O80" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P80" s="15" t="inlineStr"/>
     </row>
@@ -6905,7 +6905,7 @@
         <v>2</v>
       </c>
       <c r="O81" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P81" s="15" t="inlineStr"/>
     </row>
@@ -6977,7 +6977,7 @@
         <v>2</v>
       </c>
       <c r="O82" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P82" s="15" t="inlineStr"/>
     </row>
@@ -7049,7 +7049,7 @@
         <v>2</v>
       </c>
       <c r="O83" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P83" s="15" t="inlineStr"/>
     </row>
@@ -7121,7 +7121,7 @@
         <v>2</v>
       </c>
       <c r="O84" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P84" s="15" t="inlineStr"/>
     </row>
@@ -7193,7 +7193,7 @@
         <v>2</v>
       </c>
       <c r="O85" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P85" s="15" t="inlineStr"/>
     </row>
@@ -7265,7 +7265,7 @@
         <v>2</v>
       </c>
       <c r="O86" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P86" s="15" t="inlineStr"/>
     </row>
@@ -7337,7 +7337,7 @@
         <v>2</v>
       </c>
       <c r="O87" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P87" s="15" t="inlineStr"/>
     </row>
@@ -7409,7 +7409,7 @@
         <v>2</v>
       </c>
       <c r="O88" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P88" s="15" t="inlineStr"/>
     </row>
@@ -7481,7 +7481,7 @@
         <v>2</v>
       </c>
       <c r="O89" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P89" s="15" t="inlineStr"/>
     </row>
@@ -7553,7 +7553,7 @@
         <v>2</v>
       </c>
       <c r="O90" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P90" s="15" t="inlineStr"/>
     </row>
@@ -7625,7 +7625,7 @@
         <v>2</v>
       </c>
       <c r="O91" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P91" s="15" t="inlineStr"/>
     </row>
@@ -7697,7 +7697,7 @@
         <v>2</v>
       </c>
       <c r="O92" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P92" s="15" t="inlineStr"/>
     </row>
@@ -7769,7 +7769,7 @@
         <v>2</v>
       </c>
       <c r="O93" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P93" s="15" t="inlineStr"/>
     </row>
@@ -7841,7 +7841,7 @@
         <v>2</v>
       </c>
       <c r="O94" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P94" s="15" t="inlineStr"/>
     </row>
@@ -7913,7 +7913,7 @@
         <v>2</v>
       </c>
       <c r="O95" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P95" s="15" t="inlineStr"/>
     </row>
@@ -7985,7 +7985,7 @@
         <v>2</v>
       </c>
       <c r="O96" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P96" s="15" t="inlineStr"/>
     </row>
@@ -8057,7 +8057,7 @@
         <v>2</v>
       </c>
       <c r="O97" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P97" s="15" t="inlineStr"/>
     </row>
@@ -8129,7 +8129,7 @@
         <v>2</v>
       </c>
       <c r="O98" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P98" s="15" t="inlineStr"/>
     </row>
@@ -8201,7 +8201,7 @@
         <v>2</v>
       </c>
       <c r="O99" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P99" s="15" t="inlineStr"/>
     </row>
@@ -8273,7 +8273,7 @@
         <v>2</v>
       </c>
       <c r="O100" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P100" s="15" t="inlineStr"/>
     </row>
@@ -8345,7 +8345,7 @@
         <v>2</v>
       </c>
       <c r="O101" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P101" s="15" t="inlineStr"/>
     </row>
@@ -8417,7 +8417,7 @@
         <v>2</v>
       </c>
       <c r="O102" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P102" s="17" t="inlineStr">
         <is>
@@ -8493,7 +8493,7 @@
         <v>2</v>
       </c>
       <c r="O103" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P103" s="15" t="inlineStr"/>
     </row>
@@ -8565,7 +8565,7 @@
         <v>2</v>
       </c>
       <c r="O104" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P104" s="15" t="inlineStr"/>
     </row>
@@ -8637,7 +8637,7 @@
         <v>2</v>
       </c>
       <c r="O105" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P105" s="15" t="inlineStr"/>
     </row>
@@ -8709,7 +8709,7 @@
         <v>2</v>
       </c>
       <c r="O106" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P106" s="15" t="inlineStr"/>
     </row>
@@ -8781,7 +8781,7 @@
         <v>2</v>
       </c>
       <c r="O107" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P107" s="15" t="inlineStr"/>
     </row>
@@ -8853,7 +8853,7 @@
         <v>2</v>
       </c>
       <c r="O108" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P108" s="15" t="inlineStr"/>
     </row>
@@ -8925,7 +8925,7 @@
         <v>2</v>
       </c>
       <c r="O109" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P109" s="17" t="inlineStr">
         <is>
@@ -9001,7 +9001,7 @@
         <v>2</v>
       </c>
       <c r="O110" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P110" s="15" t="inlineStr"/>
     </row>
@@ -9073,7 +9073,7 @@
         <v>2</v>
       </c>
       <c r="O111" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P111" s="15" t="inlineStr"/>
     </row>
@@ -9145,7 +9145,7 @@
         <v>2</v>
       </c>
       <c r="O112" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P112" s="15" t="inlineStr"/>
     </row>
@@ -9217,7 +9217,7 @@
         <v>2</v>
       </c>
       <c r="O113" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P113" s="17" t="inlineStr">
         <is>
@@ -9293,7 +9293,7 @@
         <v>2</v>
       </c>
       <c r="O114" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P114" s="15" t="inlineStr"/>
     </row>
@@ -9365,7 +9365,7 @@
         <v>2</v>
       </c>
       <c r="O115" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P115" s="15" t="inlineStr"/>
     </row>
@@ -9437,7 +9437,7 @@
         <v>2</v>
       </c>
       <c r="O116" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P116" s="15" t="inlineStr"/>
     </row>
@@ -9509,7 +9509,7 @@
         <v>2</v>
       </c>
       <c r="O117" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P117" s="15" t="inlineStr"/>
     </row>
@@ -9581,7 +9581,7 @@
         <v>2</v>
       </c>
       <c r="O118" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P118" s="15" t="inlineStr"/>
     </row>
@@ -9653,7 +9653,7 @@
         <v>2</v>
       </c>
       <c r="O119" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P119" s="15" t="inlineStr"/>
     </row>
@@ -9725,7 +9725,7 @@
         <v>2</v>
       </c>
       <c r="O120" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P120" s="15" t="inlineStr"/>
     </row>
@@ -9797,7 +9797,7 @@
         <v>2</v>
       </c>
       <c r="O121" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P121" s="15" t="inlineStr"/>
     </row>
@@ -9869,7 +9869,7 @@
         <v>2</v>
       </c>
       <c r="O122" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P122" s="15" t="inlineStr"/>
     </row>
@@ -9941,7 +9941,7 @@
         <v>2</v>
       </c>
       <c r="O123" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P123" s="15" t="inlineStr"/>
     </row>
@@ -10013,7 +10013,7 @@
         <v>2</v>
       </c>
       <c r="O124" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P124" s="15" t="inlineStr"/>
     </row>
@@ -10085,7 +10085,7 @@
         <v>2</v>
       </c>
       <c r="O125" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P125" s="15" t="inlineStr"/>
     </row>
@@ -10157,7 +10157,7 @@
         <v>2</v>
       </c>
       <c r="O126" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P126" s="15" t="inlineStr"/>
     </row>
@@ -10229,7 +10229,7 @@
         <v>2</v>
       </c>
       <c r="O127" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P127" s="15" t="inlineStr"/>
     </row>
@@ -10301,7 +10301,7 @@
         <v>2</v>
       </c>
       <c r="O128" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P128" s="15" t="inlineStr"/>
     </row>
@@ -10373,7 +10373,7 @@
         <v>2</v>
       </c>
       <c r="O129" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P129" s="15" t="inlineStr"/>
     </row>
@@ -10445,7 +10445,7 @@
         <v>2</v>
       </c>
       <c r="O130" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P130" s="15" t="inlineStr"/>
     </row>
@@ -10517,7 +10517,7 @@
         <v>2</v>
       </c>
       <c r="O131" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P131" s="15" t="inlineStr"/>
     </row>
@@ -10589,7 +10589,7 @@
         <v>2</v>
       </c>
       <c r="O132" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P132" s="15" t="inlineStr"/>
     </row>
@@ -10661,7 +10661,7 @@
         <v>2</v>
       </c>
       <c r="O133" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P133" s="15" t="inlineStr"/>
     </row>
@@ -10733,7 +10733,7 @@
         <v>2</v>
       </c>
       <c r="O134" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P134" s="15" t="inlineStr"/>
     </row>
@@ -10805,7 +10805,7 @@
         <v>2</v>
       </c>
       <c r="O135" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P135" s="15" t="inlineStr"/>
     </row>
@@ -10877,7 +10877,7 @@
         <v>2</v>
       </c>
       <c r="O136" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P136" s="15" t="inlineStr"/>
     </row>
@@ -10949,7 +10949,7 @@
         <v>2</v>
       </c>
       <c r="O137" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P137" s="15" t="inlineStr"/>
     </row>
@@ -11021,7 +11021,7 @@
         <v>2</v>
       </c>
       <c r="O138" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P138" s="15" t="inlineStr"/>
     </row>
@@ -11093,7 +11093,7 @@
         <v>2</v>
       </c>
       <c r="O139" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P139" s="15" t="inlineStr"/>
     </row>
@@ -11165,7 +11165,7 @@
         <v>2</v>
       </c>
       <c r="O140" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P140" s="15" t="inlineStr"/>
     </row>
@@ -11237,7 +11237,7 @@
         <v>2</v>
       </c>
       <c r="O141" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P141" s="15" t="inlineStr"/>
     </row>
@@ -11309,7 +11309,7 @@
         <v>2</v>
       </c>
       <c r="O142" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P142" s="15" t="inlineStr"/>
     </row>
@@ -11381,7 +11381,7 @@
         <v>2</v>
       </c>
       <c r="O143" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P143" s="15" t="inlineStr"/>
     </row>
@@ -11453,7 +11453,7 @@
         <v>2</v>
       </c>
       <c r="O144" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P144" s="15" t="inlineStr"/>
     </row>
@@ -11525,7 +11525,7 @@
         <v>2</v>
       </c>
       <c r="O145" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P145" s="15" t="inlineStr"/>
     </row>
@@ -11597,7 +11597,7 @@
         <v>2</v>
       </c>
       <c r="O146" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P146" s="15" t="inlineStr"/>
     </row>
@@ -11669,7 +11669,7 @@
         <v>2</v>
       </c>
       <c r="O147" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P147" s="15" t="inlineStr"/>
     </row>
@@ -11741,7 +11741,7 @@
         <v>2</v>
       </c>
       <c r="O148" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P148" s="15" t="inlineStr"/>
     </row>
@@ -11813,7 +11813,7 @@
         <v>2</v>
       </c>
       <c r="O149" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P149" s="15" t="inlineStr"/>
     </row>
@@ -11885,7 +11885,7 @@
         <v>2</v>
       </c>
       <c r="O150" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P150" s="15" t="inlineStr"/>
     </row>
@@ -11957,7 +11957,7 @@
         <v>2</v>
       </c>
       <c r="O151" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P151" s="15" t="inlineStr"/>
     </row>
@@ -12029,7 +12029,7 @@
         <v>2</v>
       </c>
       <c r="O152" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P152" s="15" t="inlineStr"/>
     </row>
@@ -12101,7 +12101,7 @@
         <v>2</v>
       </c>
       <c r="O153" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P153" s="17" t="inlineStr">
         <is>
@@ -12177,7 +12177,7 @@
         <v>2</v>
       </c>
       <c r="O154" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P154" s="15" t="inlineStr"/>
     </row>
@@ -12249,7 +12249,7 @@
         <v>2</v>
       </c>
       <c r="O155" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P155" s="15" t="inlineStr"/>
     </row>
@@ -12321,7 +12321,7 @@
         <v>2</v>
       </c>
       <c r="O156" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P156" s="15" t="inlineStr"/>
     </row>
@@ -12393,7 +12393,7 @@
         <v>2</v>
       </c>
       <c r="O157" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P157" s="15" t="inlineStr"/>
     </row>
@@ -12465,7 +12465,7 @@
         <v>2</v>
       </c>
       <c r="O158" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P158" s="15" t="inlineStr"/>
     </row>
@@ -12537,7 +12537,7 @@
         <v>2</v>
       </c>
       <c r="O159" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P159" s="17" t="inlineStr">
         <is>
@@ -12613,7 +12613,7 @@
         <v>2</v>
       </c>
       <c r="O160" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P160" s="17" t="inlineStr">
         <is>
@@ -12689,7 +12689,7 @@
         <v>2</v>
       </c>
       <c r="O161" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P161" s="17" t="inlineStr">
         <is>
@@ -12765,7 +12765,7 @@
         <v>2</v>
       </c>
       <c r="O162" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P162" s="15" t="inlineStr"/>
     </row>
@@ -12837,7 +12837,7 @@
         <v>2</v>
       </c>
       <c r="O163" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P163" s="15" t="inlineStr"/>
     </row>
@@ -12909,7 +12909,7 @@
         <v>2</v>
       </c>
       <c r="O164" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P164" s="15" t="inlineStr"/>
     </row>
@@ -12981,7 +12981,7 @@
         <v>2</v>
       </c>
       <c r="O165" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P165" s="15" t="inlineStr"/>
     </row>
@@ -13053,7 +13053,7 @@
         <v>2</v>
       </c>
       <c r="O166" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P166" s="15" t="inlineStr"/>
     </row>
@@ -13125,7 +13125,7 @@
         <v>2</v>
       </c>
       <c r="O167" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P167" s="15" t="inlineStr"/>
     </row>
@@ -13197,7 +13197,7 @@
         <v>2</v>
       </c>
       <c r="O168" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P168" s="15" t="inlineStr"/>
     </row>
@@ -13269,7 +13269,7 @@
         <v>2</v>
       </c>
       <c r="O169" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P169" s="15" t="inlineStr"/>
     </row>
@@ -13341,7 +13341,7 @@
         <v>2</v>
       </c>
       <c r="O170" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P170" s="15" t="inlineStr"/>
     </row>
@@ -13413,7 +13413,7 @@
         <v>2</v>
       </c>
       <c r="O171" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P171" s="15" t="inlineStr"/>
     </row>
@@ -13485,7 +13485,7 @@
         <v>2</v>
       </c>
       <c r="O172" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P172" s="15" t="inlineStr"/>
     </row>
@@ -13557,7 +13557,7 @@
         <v>2</v>
       </c>
       <c r="O173" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P173" s="15" t="inlineStr"/>
     </row>
@@ -13629,7 +13629,7 @@
         <v>2</v>
       </c>
       <c r="O174" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P174" s="15" t="inlineStr"/>
     </row>
@@ -13701,7 +13701,7 @@
         <v>2</v>
       </c>
       <c r="O175" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P175" s="15" t="inlineStr"/>
     </row>
@@ -13773,7 +13773,7 @@
         <v>2</v>
       </c>
       <c r="O176" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P176" s="15" t="inlineStr"/>
     </row>
@@ -13845,7 +13845,7 @@
         <v>2</v>
       </c>
       <c r="O177" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P177" s="15" t="inlineStr"/>
     </row>
@@ -13917,7 +13917,7 @@
         <v>2</v>
       </c>
       <c r="O178" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P178" s="15" t="inlineStr"/>
     </row>
@@ -13989,7 +13989,7 @@
         <v>2</v>
       </c>
       <c r="O179" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P179" s="15" t="inlineStr"/>
     </row>
@@ -14061,7 +14061,7 @@
         <v>2</v>
       </c>
       <c r="O180" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P180" s="15" t="inlineStr"/>
     </row>
@@ -14133,7 +14133,7 @@
         <v>2</v>
       </c>
       <c r="O181" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P181" s="15" t="inlineStr"/>
     </row>
@@ -14205,7 +14205,7 @@
         <v>2</v>
       </c>
       <c r="O182" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P182" s="15" t="inlineStr"/>
     </row>
@@ -14277,7 +14277,7 @@
         <v>2</v>
       </c>
       <c r="O183" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P183" s="15" t="inlineStr"/>
     </row>
@@ -14349,7 +14349,7 @@
         <v>2</v>
       </c>
       <c r="O184" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P184" s="15" t="inlineStr"/>
     </row>
@@ -14421,7 +14421,7 @@
         <v>2</v>
       </c>
       <c r="O185" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P185" s="15" t="inlineStr"/>
     </row>
@@ -14493,7 +14493,7 @@
         <v>2</v>
       </c>
       <c r="O186" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P186" s="15" t="inlineStr"/>
     </row>
@@ -14565,7 +14565,7 @@
         <v>2</v>
       </c>
       <c r="O187" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P187" s="15" t="inlineStr"/>
     </row>
@@ -14637,7 +14637,7 @@
         <v>2</v>
       </c>
       <c r="O188" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P188" s="15" t="inlineStr"/>
     </row>
@@ -14709,7 +14709,7 @@
         <v>2</v>
       </c>
       <c r="O189" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P189" s="15" t="inlineStr"/>
     </row>
@@ -14781,7 +14781,7 @@
         <v>2</v>
       </c>
       <c r="O190" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P190" s="15" t="inlineStr"/>
     </row>
@@ -14853,7 +14853,7 @@
         <v>2</v>
       </c>
       <c r="O191" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P191" s="15" t="inlineStr"/>
     </row>
@@ -14925,7 +14925,7 @@
         <v>2</v>
       </c>
       <c r="O192" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P192" s="15" t="inlineStr"/>
     </row>
@@ -14997,7 +14997,7 @@
         <v>2</v>
       </c>
       <c r="O193" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P193" s="15" t="inlineStr"/>
     </row>
@@ -15069,7 +15069,7 @@
         <v>2</v>
       </c>
       <c r="O194" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P194" s="15" t="inlineStr"/>
     </row>
@@ -15141,7 +15141,7 @@
         <v>2</v>
       </c>
       <c r="O195" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P195" s="15" t="inlineStr"/>
     </row>
@@ -15213,7 +15213,7 @@
         <v>2</v>
       </c>
       <c r="O196" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P196" s="15" t="inlineStr"/>
     </row>
@@ -15285,7 +15285,7 @@
         <v>2</v>
       </c>
       <c r="O197" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P197" s="15" t="inlineStr"/>
     </row>
@@ -15357,7 +15357,7 @@
         <v>2</v>
       </c>
       <c r="O198" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P198" s="15" t="inlineStr"/>
     </row>
@@ -15429,7 +15429,7 @@
         <v>2</v>
       </c>
       <c r="O199" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P199" s="15" t="inlineStr"/>
     </row>
@@ -15501,7 +15501,7 @@
         <v>2</v>
       </c>
       <c r="O200" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P200" s="15" t="inlineStr"/>
     </row>
@@ -15573,7 +15573,7 @@
         <v>2</v>
       </c>
       <c r="O201" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P201" s="15" t="inlineStr"/>
     </row>
@@ -15645,7 +15645,7 @@
         <v>2</v>
       </c>
       <c r="O202" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P202" s="15" t="inlineStr"/>
     </row>
@@ -15717,7 +15717,7 @@
         <v>2</v>
       </c>
       <c r="O203" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P203" s="15" t="inlineStr"/>
     </row>
@@ -15789,7 +15789,7 @@
         <v>2</v>
       </c>
       <c r="O204" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P204" s="17" t="inlineStr">
         <is>
@@ -15865,7 +15865,7 @@
         <v>2</v>
       </c>
       <c r="O205" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P205" s="15" t="inlineStr"/>
     </row>
@@ -15937,7 +15937,7 @@
         <v>2</v>
       </c>
       <c r="O206" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P206" s="15" t="inlineStr"/>
     </row>
@@ -16009,7 +16009,7 @@
         <v>2</v>
       </c>
       <c r="O207" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P207" s="15" t="inlineStr"/>
     </row>
@@ -16081,7 +16081,7 @@
         <v>2</v>
       </c>
       <c r="O208" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P208" s="15" t="inlineStr"/>
     </row>
@@ -16153,7 +16153,7 @@
         <v>2</v>
       </c>
       <c r="O209" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P209" s="15" t="inlineStr"/>
     </row>
@@ -16225,7 +16225,7 @@
         <v>2</v>
       </c>
       <c r="O210" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P210" s="15" t="inlineStr"/>
     </row>
@@ -16297,7 +16297,7 @@
         <v>2</v>
       </c>
       <c r="O211" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P211" s="15" t="inlineStr"/>
     </row>
@@ -16369,7 +16369,7 @@
         <v>2</v>
       </c>
       <c r="O212" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P212" s="15" t="inlineStr"/>
     </row>
@@ -16441,7 +16441,7 @@
         <v>2</v>
       </c>
       <c r="O213" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P213" s="15" t="inlineStr"/>
     </row>
@@ -16513,7 +16513,7 @@
         <v>2</v>
       </c>
       <c r="O214" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P214" s="15" t="inlineStr"/>
     </row>
@@ -16585,7 +16585,7 @@
         <v>2</v>
       </c>
       <c r="O215" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P215" s="15" t="inlineStr"/>
     </row>
@@ -16657,7 +16657,7 @@
         <v>2</v>
       </c>
       <c r="O216" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P216" s="15" t="inlineStr"/>
     </row>
@@ -16729,7 +16729,7 @@
         <v>2</v>
       </c>
       <c r="O217" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P217" s="15" t="inlineStr"/>
     </row>
@@ -16801,7 +16801,7 @@
         <v>2</v>
       </c>
       <c r="O218" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P218" s="15" t="inlineStr"/>
     </row>
@@ -16873,7 +16873,7 @@
         <v>2</v>
       </c>
       <c r="O219" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P219" s="15" t="inlineStr"/>
     </row>
@@ -16945,7 +16945,7 @@
         <v>2</v>
       </c>
       <c r="O220" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P220" s="15" t="inlineStr"/>
     </row>
@@ -17017,7 +17017,7 @@
         <v>2</v>
       </c>
       <c r="O221" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P221" s="15" t="inlineStr"/>
     </row>
@@ -17089,7 +17089,7 @@
         <v>2</v>
       </c>
       <c r="O222" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P222" s="15" t="inlineStr"/>
     </row>
@@ -17161,7 +17161,7 @@
         <v>2</v>
       </c>
       <c r="O223" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P223" s="15" t="inlineStr"/>
     </row>
@@ -17233,7 +17233,7 @@
         <v>2</v>
       </c>
       <c r="O224" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P224" s="15" t="inlineStr"/>
     </row>
@@ -17305,7 +17305,7 @@
         <v>2</v>
       </c>
       <c r="O225" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P225" s="15" t="inlineStr"/>
     </row>
@@ -17377,7 +17377,7 @@
         <v>2</v>
       </c>
       <c r="O226" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P226" s="15" t="inlineStr"/>
     </row>
@@ -17449,7 +17449,7 @@
         <v>2</v>
       </c>
       <c r="O227" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P227" s="15" t="inlineStr"/>
     </row>
@@ -17521,7 +17521,7 @@
         <v>2</v>
       </c>
       <c r="O228" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P228" s="15" t="inlineStr"/>
     </row>
@@ -17593,7 +17593,7 @@
         <v>2</v>
       </c>
       <c r="O229" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P229" s="15" t="inlineStr"/>
     </row>
@@ -17665,7 +17665,7 @@
         <v>2</v>
       </c>
       <c r="O230" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P230" s="15" t="inlineStr"/>
     </row>
@@ -17737,7 +17737,7 @@
         <v>2</v>
       </c>
       <c r="O231" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P231" s="15" t="inlineStr"/>
     </row>
@@ -17809,7 +17809,7 @@
         <v>2</v>
       </c>
       <c r="O232" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P232" s="15" t="inlineStr"/>
     </row>
@@ -17881,7 +17881,7 @@
         <v>2</v>
       </c>
       <c r="O233" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P233" s="15" t="inlineStr"/>
     </row>
@@ -17953,7 +17953,7 @@
         <v>2</v>
       </c>
       <c r="O234" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P234" s="15" t="inlineStr"/>
     </row>
@@ -18025,7 +18025,7 @@
         <v>2</v>
       </c>
       <c r="O235" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P235" s="15" t="inlineStr"/>
     </row>
@@ -18097,7 +18097,7 @@
         <v>2</v>
       </c>
       <c r="O236" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P236" s="15" t="inlineStr"/>
     </row>
@@ -18169,7 +18169,7 @@
         <v>2</v>
       </c>
       <c r="O237" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P237" s="15" t="inlineStr"/>
     </row>
@@ -18241,7 +18241,7 @@
         <v>2</v>
       </c>
       <c r="O238" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P238" s="15" t="inlineStr"/>
     </row>
@@ -18313,7 +18313,7 @@
         <v>2</v>
       </c>
       <c r="O239" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P239" s="15" t="inlineStr"/>
     </row>
@@ -18385,7 +18385,7 @@
         <v>2</v>
       </c>
       <c r="O240" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P240" s="15" t="inlineStr"/>
     </row>
@@ -18457,7 +18457,7 @@
         <v>2</v>
       </c>
       <c r="O241" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P241" s="15" t="inlineStr"/>
     </row>
@@ -18529,7 +18529,7 @@
         <v>2</v>
       </c>
       <c r="O242" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P242" s="15" t="inlineStr"/>
     </row>
@@ -18601,7 +18601,7 @@
         <v>2</v>
       </c>
       <c r="O243" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P243" s="15" t="inlineStr"/>
     </row>
@@ -18673,7 +18673,7 @@
         <v>2</v>
       </c>
       <c r="O244" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P244" s="15" t="inlineStr"/>
     </row>
@@ -18745,7 +18745,7 @@
         <v>2</v>
       </c>
       <c r="O245" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P245" s="15" t="inlineStr"/>
     </row>
@@ -18817,7 +18817,7 @@
         <v>2</v>
       </c>
       <c r="O246" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P246" s="15" t="inlineStr"/>
     </row>
@@ -18889,7 +18889,7 @@
         <v>2</v>
       </c>
       <c r="O247" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P247" s="15" t="inlineStr"/>
     </row>
@@ -18961,7 +18961,7 @@
         <v>2</v>
       </c>
       <c r="O248" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P248" s="15" t="inlineStr"/>
     </row>
@@ -19033,7 +19033,7 @@
         <v>2</v>
       </c>
       <c r="O249" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P249" s="15" t="inlineStr"/>
     </row>
@@ -19105,7 +19105,7 @@
         <v>2</v>
       </c>
       <c r="O250" s="15" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="P250" s="15" t="inlineStr"/>
     </row>
@@ -19153,7 +19153,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>
@@ -21717,7 +21717,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>
@@ -24277,7 +24277,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: Kratom-eligible (FL Kratom CPA) + non-kratom SKUs   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>
@@ -26845,7 +26845,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: Kratom-eligible (TX Kratom CPA / HB 4127) + non-kratom SKUs   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: Kratom-eligible (TX Kratom CPA / HB 4127) + non-kratom SKUs   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>
@@ -29517,7 +29517,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: Kratom-eligible (TX Kratom CPA / HB 4127) + non-kratom SKUs   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: Kratom-eligible (TX Kratom CPA / HB 4127) + non-kratom SKUs   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>
@@ -32177,7 +32177,7 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Product: TBD   |   2 BAs/shift · 5.5 hrs/BA</t>
+          <t>Product: TBD   |   2 BAs/shift · 5 hrs/BA</t>
         </is>
       </c>
     </row>

</xml_diff>